<commit_message>
Add dependency tables to orch_metadata.xlsx sync workbook
Adds DependencyCondition, JobDependencies, and TaskDependencies sheets
matching orch.DependencyCondition/orch.JobDependencies/orch.TaskDependencies,
with FK-lookup dropdowns styled consistently with the existing sheets.
Existing Jobs/Tasks/ObjectIDs/TaskType records are untouched.

Also drops the stray Excel lock artifact (~$orch_metadata.xlsx) that had
been committed by accident.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VE3snD4acdGK4J2HkwA2Ay
</commit_message>
<xml_diff>
--- a/MetadataSync/orch_metadata.xlsx
+++ b/MetadataSync/orch_metadata.xlsx
@@ -10,12 +10,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TaskType" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DependencyCondition" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JobDependencies" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TaskDependencies" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="JobNameList">Jobs!$A$2:$A$1000</definedName>
     <definedName name="ObjectNameList">ObjectIDs!$B$2:$B$1000</definedName>
     <definedName name="TaskTypeList">TaskType!$A$2:$A$1000</definedName>
     <definedName name="WorkspaceNameList">ObjectIDs!$A$2:$A$1000</definedName>
+    <definedName name="DependencyConditionList">DependencyCondition!$A$2:$A$1000</definedName>
+    <definedName name="TaskNameList">Tasks!$A$2:$A$1000</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -39,7 +44,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -70,6 +75,21 @@
         <bgColor rgb="FF548235"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF375623"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -83,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -97,6 +117,9 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -478,6 +501,40 @@
     <tableColumn id="12" name="System"/>
     <tableColumn id="13" name="Layer"/>
     <tableColumn id="14" name="LoggingLevel"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblDependencyCondition" displayName="tblDependencyCondition" ref="A1:A4" headerRowCount="1">
+  <autoFilter ref="A1:A4"/>
+  <tableColumns count="1">
+    <tableColumn id="1" name="DependencyCondition"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblJobDependencies" displayName="tblJobDependencies" ref="A1:C1" headerRowCount="1">
+  <autoFilter ref="A1:C1"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="JobName"/>
+    <tableColumn id="2" name="DependentJobName"/>
+    <tableColumn id="3" name="DependsOn"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblTaskDependencies" displayName="tblTaskDependencies" ref="A1:C1" headerRowCount="1">
+  <autoFilter ref="A1:C1"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="TaskName"/>
+    <tableColumn id="2" name="DependentTaskName"/>
+    <tableColumn id="3" name="DependsOn"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2692,4 +2749,152 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>DependencyCondition</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Succeeded</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23.90625" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>JobName</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>DependentJobName</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>DependsOn</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>JobNameList</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>JobNameList</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>DependencyConditionList</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32.26953125" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>TaskName</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>DependentTaskName</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>DependsOn</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>TaskNameList</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>TaskNameList</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>DependencyConditionList</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Register the Ingest_ContosoDW_Bronze job in orch.ObjectIDs
FK_Tasks_ObjectIDs_Job requires that every Task's (WorkspaceName, JobName)
also exist as a (WorkspaceName, ObjectName) row in orch.ObjectIDs. That
row was missing for the only job currently defined, so every Task upsert
in nb_Metadata_Sync's push_excel_to_metadata failed with a FOREIGN KEY
violation on that constraint.

Added the row using the same PENDING_DEPLOYMENT_REPLACE_ME_<name>
placeholder convention already used for the two existing ObjectIDs
entries; nb_RefreshObjectIDs presumably fills in the real deployed
artifact ID later.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VE3snD4acdGK4J2HkwA2Ay
</commit_message>
<xml_diff>
--- a/MetadataSync/orch_metadata.xlsx
+++ b/MetadataSync/orch_metadata.xlsx
@@ -440,7 +440,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblObjectIDs" displayName="tblObjectIDs" ref="A1:D3" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblObjectIDs" displayName="tblObjectIDs" ref="A1:D4" headerRowCount="1">
   <autoFilter ref="A1:D2"/>
   <tableColumns count="4">
     <tableColumn id="1" name="WorkspaceName"/>
@@ -830,7 +830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="19.7265625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -900,6 +900,28 @@
         </is>
       </c>
       <c r="D3" t="inlineStr">
+        <is>
+          <t>a937b42f-1407-41c9-b5bf-33288dc7f60f</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MDF_CentralHub</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ingest_ContosoDW_Bronze</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PENDING_DEPLOYMENT_REPLACE_ME_Ingest_ContosoDW_Bronze</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>a937b42f-1407-41c9-b5bf-33288dc7f60f</t>
         </is>

</xml_diff>

<commit_message>
Fix orch_metadata.xlsx: give JobDependencies/TaskDependencies >= 1 data row
Excel silently strips a Table object whose range is only the header row
(no data rows beneath it) on open -- confirmed by the repair log naming
exactly table6.xml/table7.xml (tblJobDependencies/tblTaskDependencies),
the only two tables in the workbook with zero data rows.

Extended both tables' ref (and matching autoFilter ref) to include one
blank data row, matching the "a table needs >= 1 data row" rule the
notebook's own _write_table_rows already follows. _read_table_rows
already skips fully-blank rows, so this doesn't add a phantom row to
either orch table on push. No other data changed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VE3snD4acdGK4J2HkwA2Ay
</commit_message>
<xml_diff>
--- a/MetadataSync/orch_metadata.xlsx
+++ b/MetadataSync/orch_metadata.xlsx
@@ -517,8 +517,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblJobDependencies" displayName="tblJobDependencies" ref="A1:C1" headerRowCount="1">
-  <autoFilter ref="A1:C1"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblJobDependencies" displayName="tblJobDependencies" ref="A1:C2" headerRowCount="1">
+  <autoFilter ref="A1:C2"/>
   <tableColumns count="3">
     <tableColumn id="1" name="JobName"/>
     <tableColumn id="2" name="DependentJobName"/>
@@ -529,8 +529,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblTaskDependencies" displayName="tblTaskDependencies" ref="A1:C1" headerRowCount="1">
-  <autoFilter ref="A1:C1"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblTaskDependencies" displayName="tblTaskDependencies" ref="A1:C2" headerRowCount="1">
+  <autoFilter ref="A1:C2"/>
   <tableColumns count="3">
     <tableColumn id="1" name="TaskName"/>
     <tableColumn id="2" name="DependentTaskName"/>

</xml_diff>

<commit_message>
Populate orch.Jobs.WorkspaceName for Ingest_ContosoDW_Bronze
nb_RefreshObjectIDs' discover_object_refs() only picks up a job
(WHERE WorkspaceName IS NOT NULL) -- with this column empty, the job
was silently excluded from every refresh, so orch.ObjectIDs would
never get past its PENDING_DEPLOYMENT_REPLACE_ME placeholder for it
no matter how many times the notebook ran.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VE3snD4acdGK4J2HkwA2Ay
</commit_message>
<xml_diff>
--- a/MetadataSync/orch_metadata.xlsx
+++ b/MetadataSync/orch_metadata.xlsx
@@ -1084,6 +1084,11 @@
       <c r="E2" t="n">
         <v>60</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>MDF_CentralHub</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>DEV</t>

</xml_diff>

<commit_message>
Correct all WorkspaceName values in orch_metadata.xlsx to Wave MDF CentralHub
ObjectIDs (3 rows), Jobs (1 row), and Tasks (27 rows) all had
WorkspaceName = "MDF_CentralHub" -- this repo's folder name, not the
actual Fabric workspace display name ("Wave MDF CentralHub"). No other
cell values touched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VE3snD4acdGK4J2HkwA2Ay
</commit_message>
<xml_diff>
--- a/MetadataSync/orch_metadata.xlsx
+++ b/MetadataSync/orch_metadata.xlsx
@@ -864,7 +864,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -886,7 +886,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -908,7 +908,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>MDF_CentralHub</t>
+          <t>Wave MDF CentralHub</t>
         </is>
       </c>
       <c r="F28" t="n">

</xml_diff>